<commit_message>
Update outreach-tracker.xlsx after batch outreach run 2026-03-24
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -524,6 +524,816 @@
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Risk Management Institution of Australasia</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RMIA</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>rmia.org.au</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Risk Management</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Simon Levy</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>simon.levy@rmia.org.au</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Communication and Public Relations Australia</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CPRA</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>cpra.org.au</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Communications/PR</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Louise Harland-Cox</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>louise@cpra.org.au</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Formerly PRIA, rebranded Feb 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Planning Institute of Australia</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PIA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>planning.org.au</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Urban Planning</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Matt Collins</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>matt.collins@planning.org.au</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>National Electrical and Communications Association</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>NECA</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>neca.asn.au</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Electrical/Communications</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Oliver Judd</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>oliver.judd@neca.asn.au</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Financial Services Institute of Australasia</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Finsia</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>finsia.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Financial Services</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Joanne Becker</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Acting GM</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>j.becker@finsia.com</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>CEO departed Sep 2025, Joanne is Acting GM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Australian Information Industry Association</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AIIA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>aiia.com.au</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Technology/IT</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Simon Bush</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>simon@aiia.com.au</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>R1W1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Institute of Finance Professionals NZ</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>INFINZ</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>infinz.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Finance</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Jim McElwain</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Executive Director</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>jim@infinz.com</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>New Zealand Events Association</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>NZEA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>nzea.co</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Elaine Linnell</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>elaine@nzea.co</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1000+ members</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Infrastructure New Zealand</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>InfraNZ</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>infrastructure.org.nz</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Infrastructure</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Nick Leggett</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>nick.leggett@infrastructure.org.nz</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Email format confirmed from predecessor</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Employers and Manufacturers Association</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>EMA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ema.co.nz</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Business/Employers</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>John Fraser-Mackenzie</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>john.fraser-mackenzie@ema.co.nz</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Email format confirmed from predecessor brett.oriley@</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Marketing Association of New Zealand</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MANZ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>marketing.org.nz</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>John Miles</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>john@marketing.org.nz</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>BusinessNZ</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>BNZ</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>businessnz.org.nz</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Business Advocacy</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>info@businessnz.org.nz</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>R1W2</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Generic inbox, no direct CEO email found</t>
         </is>
       </c>
     </row>
@@ -587,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -648,6 +1458,84 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>W1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in Australia</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>First wave - all direct CEO emails</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>W2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in New Zealand</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>NZ associations - 5 direct CEO emails, 1 generic</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update batch outreach Run 2: 66 drafts across 11 waves
Adds state-level associations (NSW, VIC, QLD, WA, SA, TAS, ACT, NT) and
NSW conference producers. Running total: 66 drafts this run.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -986,13 +986,11 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
           <t>R1W2</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1053,7 +1051,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
           <t>R1W2</t>
@@ -1124,7 +1121,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
           <t>R1W2</t>
@@ -1195,7 +1191,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
           <t>R1W2</t>
@@ -1266,13 +1261,11 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
           <t>R1W2</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1298,8 +1291,6 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>info@businessnz.org.nz</t>
@@ -1325,7 +1316,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
           <t>R1W2</t>
@@ -1334,6 +1324,4463 @@
       <c r="O13" t="inlineStr">
         <is>
           <t>Generic inbox, no direct CEO email found</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ASN Events</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ASN</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>asn.events</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Tim Hancock</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>tim.h@asnevents.net.au</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Email confirmed from ASN Events contact page</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>The Production House Events</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>TPHE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>theproductionhouseevents.com.au</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Harry Samuels (CEO)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>info@tphe.com.au</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>No individual emails published. Gina Samuels is Director.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>The Conference Group</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TCG</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>theconferencegroup.com.au</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Amber Anderson</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>info@theconferencegroup.com.au</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Paul Anderson is Strategic Project Lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Catalyst Event Solutions</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Catalyst</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>catalystevents.com.au</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Sarah Dixon</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Founding Director</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>info@catalystevents.com.au</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Boutique PCO based in Artarmon NSW</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Lateral Events</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Lateral</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>lateralevents.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Megan Peters</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CEO + Director</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>hello@lateralevents.com</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>30 years in industry, multi-award winning</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Alive Events Agency</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Alive</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>aliveeventsagency.com.au</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Events/Activations</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Antony Hampel</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>newbiz@a-live.com.au</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>R2W1</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Sydney/Melbourne/Byron Bay offices</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>The Conference Company</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>TCC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>theconferencecompany.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Thea Farrant Adam</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>hello@theconferencecompany.com</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Acquired by Uno Loco Group Mar 2025. Jan Tonkin is Founder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Lime Events</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Lime</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>limeevents.co.nz</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>info@limeevents.co.nz</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>BEIA Approved PCO, Auckland based</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Conferences &amp; Events Ltd</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>C&amp;E</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>confer.co.nz</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Drew Matheson</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>drew@confer.co.nz</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Email format inferred from janet@confer.co.nz (Founder)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Composition NZ</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Composition</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>composition.co.nz</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>getintouch@composition.co.nz</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Christchurch and Auckland offices</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PPG Events</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ppgevents.co.nz</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Angela Morgan</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>GM Client Operations</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>info@ppgevents.co.nz</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Auckland and Queenstown offices</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CD Event Management</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CDEM</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>cdem.co.nz</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Conference Production</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Shelley Cunningham</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>shelley@cdem.co.nz</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>R2W2</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>BEIA Approved PCO, Auckland based</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ClubsNSW</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ClubsNSW</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>clubsnsw.com.au</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Clubs/Hospitality</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Rebecca Riant</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>info@clubsnsw.com.au</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>1200+ member clubs</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of NSW</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>REINSW</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>reinsw.com.au</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Tim McKibbin</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>info@reinsw.com.au</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Peak body for RE professionals in NSW</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>NSW Farmers</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>NSWFarmers</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>nswfarmers.org.au</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Pete Arkle</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>member@nswfarmers.org.au</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Largest state farming organisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>NSW Tourism Association</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>NSWTA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>nswtourismassociation.com.au</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Natalie Godward</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>admin@nswtourismassociation.com.au</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Peak body for visitor economy in NSW</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LG Professionals NSW</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>LGPNSW</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>lgprofessionals.com.au</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Local Government</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Vicki Mayo</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>vicki@lgprofessionals.com.au</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Email format confirmed: firstname@domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Business NSW</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>BNSW</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>businessnsw.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Business/Chamber</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Daniel Hunter</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>contactus@businessnsw.com</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>R2W3</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Formerly NSW Business Chamber</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of Victoria</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>REIV</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>reiv.com.au</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Toby Balazs</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>reiv@reiv.com.au</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Victorian Farmers Federation</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>VFF</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>vff.org.au</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Charlie Thomas</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>vff@vff.org.au</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Victorian Tourism Industry Council</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>VTIC</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>vtic.com.au</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Felicia Mariani</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>info@vtic.com.au</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Victorian Healthcare Association</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>VHA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>vha.org.au</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Leigh Clarke</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>vha@vha.org.au</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Victorian TAFE Association</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>VTA</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>vta.vic.edu.au</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Education/TAFE</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Alex White</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>alex@vta.vic.edu.au</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Email format: firstname@domain</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Master Builders Victoria</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>MBV</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>mbav.com.au</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Michaela Lihou</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>mbassist@mbav.com.au</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Draft Created</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>R2W4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of Queensland</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>REIQ</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>reiq.com.au</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Antonia Mercorella</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>reception@reiq.com.au</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>2</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Queensland Tourism Industry Council</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>QTIC</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>qtic.com.au</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Brett Fraser</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>info@qtic.com.au</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>2</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Queensland Resources Council</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>QRC</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>qrc.org.au</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Resources/Mining</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Lianne Ede</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>info@qrc.org.au</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>2</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Queensland Trucking Association</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>QTA</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>qta.com.au</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Transport</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>info@qta.com.au</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>2</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Queensland Nurses and Midwives' Union</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>QNMU</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>qnmu.org.au</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>info@qnmu.org.au</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>2</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AgForce Queensland</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>AgForce</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>agforceqld.org.au</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>reception@agforceqld.org.au</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>2</v>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>QLD associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of Western Australia</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>REIWA</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>reiwa.com.au</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Blaine Slater</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>infoservice@reiwa.com.au</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>2</v>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Tourism Council WA</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>TCWA</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>tourismcouncilwa.com.au</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Evan Hall</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>tcwa@tourismcouncilwa.com.au</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>2</v>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>WAFarmers</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>WAFarmers</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>wafarmers.org.au</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Trevor Whittington</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>ceo@wafarmers.org.au</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>2</v>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Western Australian Council of Social Service</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>WACOSS</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>wacoss.org.au</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Community Services</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Louise Giolitto</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>louise@wacoss.org.au</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>2</v>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LG Professionals WA</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>LGPWA</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>lgprofessionalswa.org.au</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Local Government</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Stacey Hutt</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>stacey.hutt@lgprofessionalswa.org.au</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>2</v>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Australian Hotels Association WA</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>AHA WA</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>ahawa.asn.au</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Bradley Woods</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>exec@ahawa.asn.au</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>2</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>WA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Business SA (SA Business Chamber)</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Business SA</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>sabusinesschamber.com.au</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Business/Commerce</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Andrew Kay</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>customerservice@sabusinesschamber.com.au</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>2</v>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>South Australian Council of Social Service</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SACOSS</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>sacoss.org.au</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Community Services</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Dr Catherine Earl</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>sacoss@sacoss.org.au</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>2</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Tourism Industry Council South Australia</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>TiCSA</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>ticsa.com.au</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Shaun de Bruyn</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>info@ticsa.com.au</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>2</v>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of South Australia</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>REISA</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>reisa.com.au</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Andrea Heading</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>reisa@reisa.com.au</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>2</v>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Primary Producers SA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PPSA</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>ppsa.org.au</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Caroline Rhodes</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>admin@ppsa.org.au</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>2</v>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Local Government Association of South Australia</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LGA SA</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>lga.sa.gov.au</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Local Government</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Matt Pinnegar</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>lgasa@lga.sa.gov.au</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>SA associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Tasmanian Chamber of Commerce and Industry</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>TCCI</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>tcci.com.au</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Business/Commerce</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Michael Bailey OAM</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>admin@tcci.com.au</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>2</v>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of Tasmania</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>REIT</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>reit.com.au</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Michelle Tynan</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>michelle.tynan@reit.com.au</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>2</v>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Tourism Industry Council Tasmania</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>TICT</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>tict.com.au</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Amy Hills</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>info@tict.com.au</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>2</v>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Tasmanian Farmers and Graziers Association</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>TFGA</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>tfga.com.au</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Nathan Calman</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>reception@tfga.com.au</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>2</v>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Tasmanian Council of Social Service</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>TasCOSS</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>tascoss.org.au</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Community Services</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Adrienne Picone</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>adrienne@tascoss.org.au</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>2</v>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Local Government Association of Tasmania</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>LGAT</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>lgat.tas.gov.au</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Local Government</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Dion Lester</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>admin@lgat.tas.gov.au</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>2</v>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>TAS associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Canberra Business Chamber</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>CBC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>canberrabusiness.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Business/Commerce</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Greg Harford</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>info@canberrabusiness.com</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>2</v>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Real Estate Institute of the ACT</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>REIACT</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>reiact.com.au</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Maria Edwards</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>reception@reiact.com.au</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>2</v>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Master Builders ACT</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>MBA ACT</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>mba.org.au</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Anna Neelagama</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>canberra@mba.org.au</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>2</v>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Australian Hotels Association ACT</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>AHA ACT</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>actaha.org.au</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>gm@actaha.org.au</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>2</v>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Canberra Region Tourism Leaders Forum</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>CRTLF</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>tlforum.com.au</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>David Marshall</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Chair</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>admin@tlforum.com.au</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>2</v>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ClubsACT</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>ClubsACT</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>clubsact.com.au</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Clubs/Hospitality</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Craig Shannon</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>info@clubsact.com.au</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>2</v>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>ACT associations</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Chamber of Commerce NT</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>CCNT</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>chambernt.com.au</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Business/Commerce</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Glen Hingley</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>ceo@chambernt.com.au</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>2</v>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Tourism Top End</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>TTE</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>tourismtopend.com.au</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Samantha Bennett</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>GM</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>gm@tourismtopend.com.au</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>2</v>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Real Estate Institute NT</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>REINT</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>reint.com.au</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Real Estate</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Jo Fitzpatrick</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>reception@reint.com.au</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>2</v>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Hospitality NT</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>HNT</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>hospitalitynt.com.au</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Hospitality</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Alexander Bruce</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>admin@hospitalitynt.com.au</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>2</v>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LGANT</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>LGANT</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>lgant.asn.au</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Local Government</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Mary Watson</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>info@lgant.asn.au</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>2</v>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>NT Farmers</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>NTF</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>ntfarmers.org.au</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Agriculture</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Andrew Bourne</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Acting CEO</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>ceo@ntfarmers.org.au</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>2</v>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>NT associations. ASBA Darwin conference reference used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Eventscape</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>eventscape.com.au</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>3</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>(Generic inbox)</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>info@eventscape.com.au</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="n">
+        <v>2</v>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ID Events Australia</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>IDEA</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ideventsaustralia.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Claire Winn</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Executive General Manager</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>idsales@ideventsaustralia.com</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="n">
+        <v>2</v>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Veritas Events</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>VE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>veritas.com.au</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Kieran Kennedy</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>create@veritas.com.au</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="n">
+        <v>2</v>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>DNA Event Management</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>DNA</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>dnaevents.com.au</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Anne Smith</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Owner &amp; Director</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>anne@dnaevents.com.au</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="n">
+        <v>2</v>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>On Purpose Events</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>OPE</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>onpurposeevents.co</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>(Generic inbox)</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>hello@onpurposeevents.co</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="n">
+        <v>2</v>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Will Organise</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>willorganise.com.au</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Conference/Events</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>3</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>(Generic inbox)</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>willorg@willorganise.com.au</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Draft created</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="n">
+        <v>2</v>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>NSW conference producers.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run 3: Research 16 conference producers across VIC, QLD, WA, SA, ACT, NT
Researched 16 new targets across 7 state conference producer segments.
Wave 1 (VIC): 6 targets including ACEO, Liberty Events, JT Production, Peanut Productions, MCO Events, FruitBowl.
Wave 2 (QLD): 5 targets including Event Society, Absolute Events, FAME Events, Glo Events, Anagram Events.
Wave 3 (WA/SA/ACT/NT): 5 targets including Event & Conference Co, Seed Events, Conference Co-ordinators, Agentur, Bask Event Management.
Status: Researched - pending Gemini for email generation.
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O79"/>
+  <dimension ref="A1:O95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5429,7 +5429,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M74" t="inlineStr"/>
       <c r="N74" t="n">
         <v>2</v>
       </c>
@@ -5498,7 +5497,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M75" t="inlineStr"/>
       <c r="N75" t="n">
         <v>2</v>
       </c>
@@ -5567,7 +5565,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M76" t="inlineStr"/>
       <c r="N76" t="n">
         <v>2</v>
       </c>
@@ -5636,7 +5633,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M77" t="inlineStr"/>
       <c r="N77" t="n">
         <v>2</v>
       </c>
@@ -5705,7 +5701,6 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M78" t="inlineStr"/>
       <c r="N78" t="n">
         <v>2</v>
       </c>
@@ -5774,13 +5769,1056 @@
           <t>2026-03-24</t>
         </is>
       </c>
-      <c r="M79" t="inlineStr"/>
       <c r="N79" t="n">
         <v>2</v>
       </c>
       <c r="O79" t="inlineStr">
         <is>
           <t>NSW conference producers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Australian Conference &amp; Event Organisers</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ACEO</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>aceo.net.au</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>3</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Mandy Bromilow</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Director/Founder</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>mandy@aceo.net.au</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>3</v>
+      </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne PCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Liberty Events</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr"/>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>libertyevents.com.au</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>3</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Kira Fitzpatrick</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>sales@libertyevents.com.au</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>3</v>
+      </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne corporate events</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>JT Production Management</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>JTPM</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>jtproductionmanagement.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>3</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Julia Truong</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>enquiries@jtproductionmanagement.com</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>3</v>
+      </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne 1200+ events</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Peanut Productions</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>peanutproductions.com.au</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>3</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Matthew Jackson</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>Head of Commercial</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>matthew@peanutproductions.com.au</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N83" t="n">
+        <v>3</v>
+      </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne/Sydney events &amp; video</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>MCO Events</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>mcoevents.com.au</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Melissa Yu</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>enquiries@mcoevents.com.au</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>3</v>
+      </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne MICE boutique agency</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>FruitBowl Events Agency</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>fruitbowl.com.au</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>3</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Tammy Crupi</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Founder/Director</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>info@fruitbowl.com.au</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N85" t="n">
+        <v>3</v>
+      </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>VIC - Melbourne 28 yrs experience</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Event Society</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>eventsociety.com.au</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Decinda Burrell</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Creative Director</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>admin@eventsociety.com.au</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N86" t="n">
+        <v>3</v>
+      </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>QLD - Brisbane/Gold Coast events</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Absolute Events &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>AEM</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>absoluteeventsandmarketing.com.au</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>3</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Susan Harris</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Managing Director &amp; Event Director</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>susan@absoluteeventsandmarketing.com.au</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N87" t="n">
+        <v>3</v>
+      </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>QLD - Brisbane PCO 18+ years</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>FAME Events</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>fame-events.com.au</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>April Booij</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Founder</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>hello@fame-events.com.au</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N88" t="n">
+        <v>3</v>
+      </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>QLD - Brisbane conference &amp; corporate</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Glo Events</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>gloevents.com.au</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>3</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Pete Cunningham</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Co-Founder</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>hello@gloevents.com.au</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N89" t="n">
+        <v>3</v>
+      </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>QLD - Brisbane event production, own venue</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Anagram Events</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr"/>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>anagramevents.com.au</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>3</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Steven Turner</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>admin@anagramevents.com.au</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N90" t="n">
+        <v>3</v>
+      </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>QLD - Brisbane tech/education conferences</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Event &amp; Conference Co</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ECC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>eventandconferenceco.com.au</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>3</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Rebecca Cole</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Director</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>hello@eventandconferenceco.com.au</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N91" t="n">
+        <v>3</v>
+      </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>WA - Perth PCO 600+ events</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Seed Events</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr"/>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>seedevents.com.au</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>(Generic inbox)</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>admin@seedevents.com.au</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N92" t="n">
+        <v>3</v>
+      </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>SA - Adelaide conferences/forums</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Conference Co-ordinators</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ConfCo</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>conferenceco.com.au</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>3</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>(Generic inbox)</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>conference@confco.com.au</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N93" t="n">
+        <v>3</v>
+      </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>ACT - Canberra PCO est. 1995</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Agentur</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr"/>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>agentur.com.au</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>3</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Britta Decker</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Managing Director</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>info@agentur.com.au</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N94" t="n">
+        <v>3</v>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>NT - Darwin full-service events</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Bask Event Management</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>baskeventmanagement.com.au</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Events</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>3</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Andrea Allen</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Owner &amp; Managing Director</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>info@baskeventmanagement.com.au</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N95" t="n">
+        <v>3</v>
+      </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>NT - Darwin sport/wellness events</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update outreach-tracker with Run 4 Wave 1 - 6 Sydney association targets
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O95"/>
+  <dimension ref="A1:O101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5852,7 +5852,6 @@
           <t>Liberty Events</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>libertyevents.com.au</t>
@@ -5984,7 +5983,6 @@
           <t>Peanut Productions</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>peanutproductions.com.au</t>
@@ -6048,7 +6046,6 @@
           <t>MCO Events</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>mcoevents.com.au</t>
@@ -6112,7 +6109,6 @@
           <t>FruitBowl Events Agency</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>fruitbowl.com.au</t>
@@ -6176,7 +6172,6 @@
           <t>Event Society</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>eventsociety.com.au</t>
@@ -6308,7 +6303,6 @@
           <t>FAME Events</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>fame-events.com.au</t>
@@ -6372,7 +6366,6 @@
           <t>Glo Events</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>gloevents.com.au</t>
@@ -6436,7 +6429,6 @@
           <t>Anagram Events</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>anagramevents.com.au</t>
@@ -6568,7 +6560,6 @@
           <t>Seed Events</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>seedevents.com.au</t>
@@ -6700,7 +6691,6 @@
           <t>Agentur</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>agentur.com.au</t>
@@ -6764,7 +6754,6 @@
           <t>Bask Event Management</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>baskeventmanagement.com.au</t>
@@ -6819,6 +6808,414 @@
       <c r="O95" t="inlineStr">
         <is>
           <t>NT - Darwin sport/wellness events</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Committee for Sydney</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>CFS</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>sydney.org.au</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Urban policy / Think tank</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>1</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Eamon Waterford</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>eamon@sydney.org.au</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N96" t="n">
+        <v>4</v>
+      </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Email inferred from colleague pattern (hannah@, matt@)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Business Events Sydney</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>BESydney</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>besydney.com.au</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Business events / Conventions</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>Amanda Lampe</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>alampe@besydney.com.au</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N97" t="n">
+        <v>4</v>
+      </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Email inferred from colleague pattern (sstewart@, knicholls@, clenehan@)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>CBD Sydney Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>CBDSCC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>cbdsydneychamber.com.au</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Chamber of commerce</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Peter May</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Executive Officer</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Peter.May@cbdsydneychamber.com.au</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N98" t="n">
+        <v>4</v>
+      </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Email from City of Sydney official listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Parramatta Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>PCC</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>parramattachamber.com.au</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Chamber of commerce</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Romina Bousimon</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>romina@parramattachamber.com.au</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N99" t="n">
+        <v>4</v>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Email from official board/team page</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Western Sydney Leadership Dialogue</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>WSLD</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>westernsydney.org.au</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Think tank / Policy</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Adam Leto</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>info@westernsydney.org.au</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>Generic</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N100" t="n">
+        <v>4</v>
+      </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Generic inbox - no direct CEO email publicly available</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Canterbury Bankstown Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>CBCC</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>cbchamber.org.au</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Chamber of commerce</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Wally Mehanna</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>ceo@cbchamber.org.au</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Direct</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="N101" t="n">
+        <v>4</v>
+      </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Role-based email confirmed from web search</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run 5: Melbourne associations research (6 targets)
Research phase for Professional and industry associations in Melbourne.
Also backfilled Sydney run4 targets to tracker.

Targets: Melbourne Convention Bureau, Manufacturing Australia,
Melbourne Royal, Yarra River Business Association, Victorian Transport
Association, VACC.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -570,6 +570,606 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Committee for Sydney</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Eamon Waterford</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>eamon@sydney.org.au</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>sydney.org.au</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Sydney's urban policy think tank and Approved Research Institute. Advocates for the whole of Sydney on issues like transport, housing, sustainability, and liveability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Business Events Sydney (BESydney)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Amanda Lampe</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>alampe@besydney.com.au</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>besydney.com.au</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Promotes Sydney as a premier destination for international business events, conventions, and incentive travel. Amanda commenced as CEO in June 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CBD Sydney Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Peter May</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Executive Officer</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Peter.May@cbdsydneychamber.com.au</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>cbdsydneychamber.com.au</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Chamber of commerce representing businesses in the Sydney CBD. Hosts networking events including After 5 Networking, Business Roundtables, and Women in Business Network.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Parramatta Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Romina Bousimon</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>General Manager</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>romina@parramattachamber.com.au</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>parramattachamber.com.au</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>One of the oldest chambers in Western Sydney. Runs the Western Sydney Awards for Business Excellence (WSABE) since 1990.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Western Sydney Leadership Dialogue</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Adam Leto</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>info@westernsydney.org.au</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>westernsydney.org.au</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Think tank established in 2015 to highlight key regional issues and spark national conversation about Greater Western Sydney.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Canterbury Bankstown Chamber of Commerce</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Wally Mehanna</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>ceo@cbchamber.org.au</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>cbchamber.org.au</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>A hub for business networking and growth, connecting local businesses across the Canterbury-Bankstown area and beyond. Established in 2016.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Melbourne Convention Bureau</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Julia Swanson</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>julia@melbournecb.com.au</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>melbournecb.com.au</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Melbourne's official convention bureau. Identifies and bids for business events and assists associations with conference bids. Julia Swanson has led MCB since 2010. Also Board Chair of BestCities Global Alliance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Manufacturing Australia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ben Eade</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ben.eade@manufacturingaustralia.com.au</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>manufacturingaustralia.com.au</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>CEO-led coalition of Australia's largest manufacturers. Works with government on regulations, innovation, trade, and energy policy. Ben Eade has been with the org since 2011.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Melbourne Royal</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Brad Jenkins</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>info@melbourneroyal.com.au</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>melbourneroyal.com.au</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Organisers of Melbourne Royal Show and managers of Melbourne Showgrounds. Heritage institution running nationally recognised awards in food, wine, beer, agriculture. Brad Jenkins CEO since 2019.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Yarra River Business Association</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Elizabeth Joldeski</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Executive Officer</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>exoff@yarrariver.melbourne</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>yarrariver.melbourne</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>One of Melbourne's longest-established business precinct associations. Represents 170+ businesses along the Yarra including Federation Square, Southgate, Crown, and WTC. Active since 1998.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Victorian Transport Association</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Peter Anderson</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>reception@vta.com.au</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>vta.com.au</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Victoria's peak freight and logistics body since 1902. Advocates to governments and regulators from the freight operator perspective. Based in Port Melbourne.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Victorian Automotive Chamber of Commerce (VACC)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Peter Jones</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>vacc@vacc.com.au</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>vacc.com.au</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Voice of Victoria's automotive industry. Supports business owners in retail, service, and repair sectors. Based in North Melbourne. Peter Jones succeeded long-serving CEO Geoff Gwilym.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -581,7 +1181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -662,6 +1262,72 @@
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>First run. Segment exhausted — virtually every AU independent school already contacted. Only Stuartholme School clean. Need next-batch.txt for new segments.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-03-24</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in Sydney</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>13</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Researched - pending Gemini</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Run 4. City-level Sydney associations. 6 substantial targets found. Many small precinct chambers skipped as volunteer-run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in Melbourne</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Researched - pending Gemini</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Run 5. City-level Melbourne associations. 6 targets found. VCCI/MCC/CfM all merged and heavily contacted. CEDA, Associations Forum, AHA Vic also previously contacted.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Brisbane associations research (Run 6) - 6 targets
Research phase for Professional and industry associations in Brisbane.
6 valid targets: Committee for Brisbane, UDIA Qld, Master Builders Qld,
QMCA, CCF Qld, QTLC. 12 orgs skipped (prior contact).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1167,6 +1167,306 @@
       <c r="K14" t="inlineStr">
         <is>
           <t>Voice of Victoria's automotive industry. Supports business owners in retail, service, and repair sectors. Based in North Melbourne. Peter Jones succeeded long-serving CEO Geoff Gwilym.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Committee for Brisbane</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jen Williams</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>admin@committeeforbrisbane.org.au</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>committeeforbrisbane.org.au</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Brisbane's leading urban policy think tank and advocacy organisation. Member-led body shaping Brisbane's future. Jen Williams CEO since June 2024, previously Executive Director of Property Council QLD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>UDIA Queensland</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kirsty Chessher-Brown</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>udia@udiaqld.com.au</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>udiaqld.com.au</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Peak industry body for urban development in Queensland. Non-profit. Kirsty Chessher-Brown CEO since Feb 2018. Represents developers, planners, and allied professionals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Master Builders Queensland</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Paul Bidwell</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>ask@mbqld.com.au</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>mbqld.com.au</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Queensland's peak building and construction association since 1882. Over 9,800 members. Paul Bidwell CEO since 2022, resigning May 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Queensland Major Contractors Association</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Andrew Chapman</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>admin@qmca.com.au</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>qmca.com.au</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Peak body for major construction and infrastructure companies in QLD. Andrew Chapman is a civil engineer with diverse project lifecycle experience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Civil Contractors Federation Queensland</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Damian Long</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ceo@ccfqld.com</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>ccfqld.com</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Peak body for civil construction in Queensland. Offices in Brisbane, Townsville, Cairns. Represents civil contractors across roads, bridges, drainage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Queensland Transport and Logistics Council</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Lauren Hewitt</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>admin@qtlc.com.au</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>qtlc.com.au</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Peak body for transport and logistics in Queensland. Based in Brisbane CBD. Represents freight, logistics, and supply chain operators.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run 7: Research 6 national Australian professional/industry associations
Segment: Professional and industry associations in Australia (national)
Targets: BCA, FSC, AFGC, FCA, COSBOA, IPA
Skipped: 20 national associations (already contacted)
Status: Researched - pending Gemini

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1470,6 +1470,306 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Business Council of Australia</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bran Black</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>comms@bca.com.au</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bca.com.au</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Australia's most prominent business advocacy group, representing CEOs of the nation's largest employers. Develops and promotes practical policies for a strong, globally competitive economy. Bran Black became Chief Executive in 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Financial Services Council</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Blake Briggs</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>info@fsc.org.au</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>fsc.org.au</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Peak body setting mandatory standards and developing policy for 100+ member companies managing $3 trillion in investments for 15.6 million Australians. Covers superannuation, life insurance, funds management, and financial advice. Blake Briggs CEO since Jan 2022.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Australian Food &amp; Grocery Council</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Colm Maguire</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>afgc@afgc.org.au</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>afgc.org.au</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Peak industry body for food, beverage, and grocery manufacturers and suppliers. Advocates to government and stakeholders on industry issues. Colm Maguire became CEO in 2025 after serving as COO. Based in Canberra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Franchise Council of Australia</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Jay Westbury</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>info@franchise.org.au</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>franchise.org.au</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Peak body for the $184 billion Australian franchise sector. Advocates for franchise businesses, provides education, and runs the annual National Franchise Convention. Jay Westbury became CEO Sep 2024, 20+ years leading peak industry bodies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Council of Small Business Organisations Australia</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Skye Cappuccio</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>info@cosboa.org.au</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>cosboa.org.au</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>National peak body representing small business interests to government. Advocates on regulation, policy, and economic conditions for 2.5 million+ small businesses. Skye Cappuccio commenced as CEO on 3 Feb 2026, previously CEO of Optometry Australia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Infrastructure Partnerships Australia</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Adrian Dwyer</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>contact@infrastructure.org.au</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>infrastructure.org.au</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Industry think tank and executive member network for social and economic infrastructure. Conducts policy research, regulatory analysis, and member events. Adrian Dwyer previously led Infrastructure Australia before joining IPA as CEO.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1481,7 +1781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1628,6 +1928,72 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>Run 5. City-level Melbourne associations. 6 targets found. VCCI/MCC/CfM all merged and heavily contacted. CEDA, Associations Forum, AHA Vic also previously contacted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in Brisbane</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Researched - pending Gemini</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Run 6. Brisbane city-level associations. 6 targets found. 12 major associations skipped due to prior contact. Only 1 CONFIRMED email (CCF Qld). Segment near exhaustion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in Australia (national)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Researched - pending Gemini</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Run 7. National-level peak bodies. 6 targets found. 20 national associations skipped — most already contacted in Mar 2026 batch outreach. All 6 targets have FALLBACK generic emails. Segment near exhaustion.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add NZ associations research (Run 8) - 6 targets
Research phase for Professional and industry associations in New Zealand.
Targets: TIA, Hospitality NZ, Retail NZ, NZGBC, Cooperative Business NZ, FGC.
5 orgs skipped (already contacted). 2 CONFIRMED, 2 HIGH, 2 FALLBACK emails.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/batch-outreach/outreach-tracker.xlsx
+++ b/data/batch-outreach/outreach-tracker.xlsx
@@ -446,7 +446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -1770,6 +1770,306 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Tourism Industry Aotearoa</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rebecca Ingram</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>rebecca.ingram@tia.org.nz</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>tia.org.nz</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>NZ's peak tourism industry body representing ~1,400 member businesses. Advocates for sustainable tourism growth, policy reform, and sector resilience. Rebecca joined as CE in March 2022 with 20+ years in tourism, marketing, and advocacy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Hospitality New Zealand</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Kristy Phillips</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>ceo@hospitality.org.nz</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>hospitality.org.nz</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>1</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>NZ's peak body for the hospitality industry, representing hotels, restaurants, cafes, and bars. Kristy Phillips appointed CE in late 2025, previously owned restaurants in Timaru for 14 years and led Barker's Foodstore &amp; Eatery venues.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Retail NZ</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Carolyn Young</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>carolyn.young@retail.kiwi</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>retail.kiwi</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CONFIRMED</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>NZ's industry association for retailers, providing advocacy, compliance advice, and professional development. Represents retailers across NZ on policy issues including employment, retail crime, and consumer trends.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>New Zealand Green Building Council</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Andrew Eagles</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>andrew.eagles@nzgbc.org.nz</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>nzgbc.org.nz</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>For-purpose nonprofit est. 2005 with 700+ members across building and construction. Develops green building rating tools, campaigns for regulatory reform, and provides sustainability education.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Cooperative Business New Zealand</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Saya Wahrlich</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>CEO</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>info@nz.coop</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>nz.coop</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Peak body for cooperatives, mutuals, and member-owned businesses in Aotearoa NZ. Advocates to government, regulators, and policymakers. Published The NZ Cooperative Economy Report 2025.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>New Zealand Food &amp; Grocery Council</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Raewyn Bleakley</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Chief Executive</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>admin@fgc.org.nz</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>fgc.org.nz</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>FALLBACK</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Researched</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Peak body representing NZ's food and grocery suppliers. Advocates on regulation, sustainability, and trade issues for the FMCG sector. Raewyn Bleakley appointed CE in October 2022.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1781,7 +2081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1994,6 +2294,39 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>Run 7. National-level peak bodies. 6 targets found. 20 national associations skipped — most already contacted in Mar 2026 batch outreach. All 6 targets have FALLBACK generic emails. Segment near exhaustion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Professional and industry associations in New Zealand</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>5 (BusinessNZ, IoD NZ, Infrastructure NZ, Property Council NZ, Civil Contractors NZ)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Researched - pending Gemini</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Run 8. NZ national associations. 2 CONFIRMED emails (TIA, Retail NZ), 2 HIGH (Hospitality NZ role-based CEO email, NZGBC inferred from colleague pattern), 2 FALLBACK generic inboxes (Cooperative Business NZ, FGC). Gemini should verify CEO direct emails for FALLBACK targets.</t>
         </is>
       </c>
     </row>

</xml_diff>